<commit_message>
Final submission: complete project with enrichment, validation, forecasts, and dashboard
</commit_message>
<xml_diff>
--- a/data/processed/ethiopia_fi_unified_data_enriched.xlsx
+++ b/data/processed/ethiopia_fi_unified_data_enriched.xlsx
@@ -5288,10 +5288,8 @@
           <t>agents_per_10k</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>2024-06-30</t>
-        </is>
+      <c r="L45" s="1" t="n">
+        <v>45473</v>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
@@ -5334,7 +5332,7 @@
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="AG45" t="inlineStr"/>
@@ -5391,10 +5389,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
+      <c r="L46" s="1" t="n">
+        <v>45657</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -5437,7 +5433,7 @@
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="AG46" t="inlineStr"/>
@@ -5476,10 +5472,8 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>2023-12-01</t>
-        </is>
+      <c r="L47" s="1" t="n">
+        <v>45261</v>
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
@@ -5522,7 +5516,7 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr"/>
@@ -5607,7 +5601,7 @@
       </c>
       <c r="AF48" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="AG48" t="inlineStr"/>
@@ -5650,10 +5644,8 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>2024-06-30</t>
-        </is>
+      <c r="L49" s="1" t="n">
+        <v>45473</v>
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
@@ -5696,7 +5688,7 @@
       </c>
       <c r="AF49" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="AG49" t="inlineStr"/>

</xml_diff>